<commit_message>
RNAi with selected rnap-i features
</commit_message>
<xml_diff>
--- a/xgb_RNAi_best_params.xlsx
+++ b/xgb_RNAi_best_params.xlsx
@@ -425,41 +425,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>subsample</t>
-        </is>
+      <c r="A1" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>n_estimators</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>max_depth</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>learning_rate</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>gamma</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>colsample_bytree</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>scores</t>
         </is>
@@ -467,117 +440,92 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="n">
-        <v>199</v>
-      </c>
-      <c r="C2" t="n">
-        <v>32</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.06667333333333332</v>
-      </c>
-      <c r="E2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0.5704844444444445</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.3231060229524245</v>
+        <v>9</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>max_depth</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>866</v>
-      </c>
-      <c r="C3" t="n">
-        <v>27</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.06667333333333332</v>
-      </c>
-      <c r="E3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0.4618207407407408</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0.322957073487192</v>
+        <v>0.414391711334597</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>learning_rate</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="n">
-        <v>199</v>
-      </c>
-      <c r="C4" t="n">
-        <v>21</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.07780888888888887</v>
-      </c>
-      <c r="E4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" t="n">
-        <v>0.4074888888888889</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.3304334240713732</v>
+        <v>197</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>n_estimators</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="n">
-        <v>2333</v>
-      </c>
-      <c r="C5" t="n">
-        <v>24</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0.1111222222222222</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>0.4074888888888889</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0.3223396639550434</v>
+        <v>5</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>min_child_weight</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.8148148148148149</v>
-      </c>
-      <c r="B6" t="n">
-        <v>2769</v>
-      </c>
-      <c r="C6" t="n">
-        <v>50</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0.2848337918871252</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0.6297555555555556</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0.328586269637507</v>
+        <v>0.3037810968767726</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>gamma</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>0.7279973494407236</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>subsample</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>0.7613173724336442</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>colsample_bytree</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>0.3790722609469879</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>reg_alpha</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>0.7399010065269028</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>reg_lambda</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added the rnafold features to the RNAi pipeline, ran with scores and new RNAi explainability
</commit_message>
<xml_diff>
--- a/xgb_RNAi_best_params.xlsx
+++ b/xgb_RNAi_best_params.xlsx
@@ -425,14 +425,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n">
-        <v>0</v>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>subsample</t>
+        </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>n_estimators</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>max_depth</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>learning_rate</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>gamma</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>colsample_bytree</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>scores</t>
         </is>
@@ -440,92 +467,117 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>9</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>max_depth</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="B2" t="n">
+        <v>199</v>
+      </c>
+      <c r="C2" t="n">
+        <v>32</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.06667333333333332</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.5704844444444445</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.3231060229524245</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.414391711334597</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>learning_rate</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>866</v>
+      </c>
+      <c r="C3" t="n">
+        <v>27</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.06667333333333332</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.4618207407407408</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.322957073487192</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>197</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>n_estimators</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="B4" t="n">
+        <v>199</v>
+      </c>
+      <c r="C4" t="n">
+        <v>21</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.07780888888888887</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.4074888888888889</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.3304334240713732</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5</v>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>min_child_weight</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="B5" t="n">
+        <v>2333</v>
+      </c>
+      <c r="C5" t="n">
+        <v>24</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.1111222222222222</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.4074888888888889</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.3223396639550434</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.3037810968767726</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>gamma</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>0.7279973494407236</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>subsample</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>0.7613173724336442</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>colsample_bytree</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>0.3790722609469879</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>reg_alpha</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>0.7399010065269028</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>reg_lambda</t>
-        </is>
+        <v>0.8148148148148149</v>
+      </c>
+      <c r="B6" t="n">
+        <v>2769</v>
+      </c>
+      <c r="C6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.2848337918871252</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.6297555555555556</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.328586269637507</v>
       </c>
     </row>
   </sheetData>

</xml_diff>